<commit_message>
feat: enhance exportCarExcel method to include detailed approval status and dates in the Excel report
</commit_message>
<xml_diff>
--- a/public/tamplate-xlsx/Tamplate_CAR Audit 2025.xlsx
+++ b/public/tamplate-xlsx/Tamplate_CAR Audit 2025.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ict\www-wsl\qms\public\tamplate-xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\qems-grace\public\tamplate-xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37707F02-C6E6-4B5F-AAEE-200C46B7D978}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE866F33-CC5A-421F-8064-7539F70323C9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,7 +54,7 @@
     <definedName name="Excel_BuiltIn_Print_Area_8">#REF!</definedName>
     <definedName name="Excel_BuiltIn_Print_Area_9" localSheetId="0">#REF!</definedName>
     <definedName name="Excel_BuiltIn_Print_Area_9">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Departement 1'!$A$1:$I$57</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Departement 1'!$A$1:$I$59</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="56">
   <si>
     <t xml:space="preserve">       Surveillance </t>
   </si>
@@ -265,6 +265,12 @@
       </rPr>
       <t>www.adyawinsa.com</t>
     </r>
+  </si>
+  <si>
+    <t>(Tanggal)</t>
+  </si>
+  <si>
+    <t>(Status)</t>
   </si>
 </sst>
 </file>
@@ -1012,19 +1018,6 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -1124,6 +1117,19 @@
         <color indexed="64"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1131,7 +1137,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="170">
+  <cellXfs count="179">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
@@ -1150,15 +1156,39 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1177,6 +1207,87 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1303,16 +1414,16 @@
     <xf numFmtId="15" fontId="1" fillId="0" borderId="50" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="53" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="54" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="55" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="53" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="55" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="52" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="54" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1375,192 +1486,144 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="41" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="41" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="55" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="56" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="59" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="60" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="57" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="58" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="41" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="61" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="41" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="41" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="52" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="56" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="57" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="60" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="61" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="58" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="59" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="41" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1594,40 +1657,10 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1826,13 +1859,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>729478</xdr:colOff>
-      <xdr:row>53</xdr:row>
+      <xdr:row>55</xdr:row>
       <xdr:rowOff>45254</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>895539</xdr:colOff>
-      <xdr:row>53</xdr:row>
+      <xdr:row>55</xdr:row>
       <xdr:rowOff>262759</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2006,13 +2039,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>1068079</xdr:colOff>
-      <xdr:row>51</xdr:row>
+      <xdr:row>52</xdr:row>
       <xdr:rowOff>604666</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>1213923</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>124536</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2380,7 +2413,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.140625" style="1" customWidth="1"/>
@@ -2900,377 +2933,377 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13"/>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="158" t="s">
+      <c r="A1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="159"/>
-      <c r="F1" s="164" t="s">
+      <c r="E1" s="28"/>
+      <c r="F1" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="G1" s="165"/>
-      <c r="H1" s="165"/>
-      <c r="I1" s="166"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="49"/>
+      <c r="I1" s="50"/>
     </row>
     <row r="2" spans="1:9" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="160"/>
-      <c r="E2" s="161"/>
-      <c r="F2" s="164"/>
-      <c r="G2" s="165"/>
-      <c r="H2" s="165"/>
-      <c r="I2" s="166"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="50"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="160"/>
-      <c r="E3" s="161"/>
-      <c r="F3" s="164"/>
-      <c r="G3" s="165"/>
-      <c r="H3" s="165"/>
-      <c r="I3" s="166"/>
+      <c r="A3" s="23"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="50"/>
     </row>
     <row r="4" spans="1:9" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="160"/>
-      <c r="E4" s="161"/>
-      <c r="F4" s="164"/>
-      <c r="G4" s="165"/>
-      <c r="H4" s="165"/>
-      <c r="I4" s="166"/>
+      <c r="A4" s="23"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="49"/>
+      <c r="H4" s="49"/>
+      <c r="I4" s="50"/>
     </row>
     <row r="5" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="15"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="160"/>
-      <c r="E5" s="161"/>
-      <c r="F5" s="167"/>
-      <c r="G5" s="168"/>
-      <c r="H5" s="168"/>
-      <c r="I5" s="169"/>
+      <c r="A5" s="23"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="53"/>
     </row>
     <row r="6" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="15"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="160"/>
-      <c r="E6" s="161"/>
+      <c r="A6" s="23"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="30"/>
       <c r="F6" s="6" t="s">
         <v>30</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="54" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="20"/>
+      <c r="I6" s="55"/>
     </row>
     <row r="7" spans="1:9" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="160"/>
-      <c r="E7" s="161"/>
-      <c r="F7" s="25" t="s">
+      <c r="A7" s="23"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="G7" s="27" t="s">
+      <c r="G7" s="62" t="s">
         <v>39</v>
       </c>
-      <c r="H7" s="21" t="s">
+      <c r="H7" s="56" t="s">
         <v>40</v>
       </c>
-      <c r="I7" s="22"/>
+      <c r="I7" s="57"/>
     </row>
     <row r="8" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="17"/>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="162"/>
-      <c r="E8" s="163"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="24"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="63"/>
+      <c r="H8" s="58"/>
+      <c r="I8" s="59"/>
     </row>
     <row r="9" spans="1:9" ht="8.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="29"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="33" t="s">
+      <c r="B9" s="64"/>
+      <c r="C9" s="65"/>
+      <c r="D9" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="E9" s="34"/>
-      <c r="F9" s="33" t="s">
+      <c r="E9" s="69"/>
+      <c r="F9" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="G9" s="34"/>
-      <c r="H9" s="37" t="s">
+      <c r="G9" s="69"/>
+      <c r="H9" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="38"/>
+      <c r="I9" s="73"/>
     </row>
     <row r="10" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="31"/>
-      <c r="B10" s="31"/>
-      <c r="C10" s="32"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="36"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="40"/>
+      <c r="A10" s="66"/>
+      <c r="B10" s="66"/>
+      <c r="C10" s="67"/>
+      <c r="D10" s="70"/>
+      <c r="E10" s="71"/>
+      <c r="F10" s="70"/>
+      <c r="G10" s="71"/>
+      <c r="H10" s="74"/>
+      <c r="I10" s="75"/>
     </row>
     <row r="11" spans="1:9" ht="6.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="41" t="s">
+      <c r="A11" s="76" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="42"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="21" t="s">
+      <c r="B11" s="77"/>
+      <c r="C11" s="78"/>
+      <c r="D11" s="56" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="48"/>
-      <c r="F11" s="133" t="s">
+      <c r="E11" s="83"/>
+      <c r="F11" s="156" t="s">
         <v>35</v>
       </c>
-      <c r="G11" s="134"/>
-      <c r="H11" s="53" t="s">
+      <c r="G11" s="157"/>
+      <c r="H11" s="88" t="s">
         <v>4</v>
       </c>
-      <c r="I11" s="53" t="s">
+      <c r="I11" s="88" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="44"/>
-      <c r="B12" s="44"/>
-      <c r="C12" s="45"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="50"/>
-      <c r="F12" s="135"/>
-      <c r="G12" s="136"/>
-      <c r="H12" s="54"/>
-      <c r="I12" s="54"/>
+      <c r="A12" s="79"/>
+      <c r="B12" s="79"/>
+      <c r="C12" s="80"/>
+      <c r="D12" s="84"/>
+      <c r="E12" s="85"/>
+      <c r="F12" s="158"/>
+      <c r="G12" s="159"/>
+      <c r="H12" s="89"/>
+      <c r="I12" s="89"/>
     </row>
     <row r="13" spans="1:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="44"/>
-      <c r="B13" s="44"/>
-      <c r="C13" s="45"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="50"/>
-      <c r="F13" s="135"/>
-      <c r="G13" s="136"/>
-      <c r="H13" s="55"/>
-      <c r="I13" s="58"/>
+      <c r="A13" s="79"/>
+      <c r="B13" s="79"/>
+      <c r="C13" s="80"/>
+      <c r="D13" s="84"/>
+      <c r="E13" s="85"/>
+      <c r="F13" s="158"/>
+      <c r="G13" s="159"/>
+      <c r="H13" s="90"/>
+      <c r="I13" s="93"/>
     </row>
     <row r="14" spans="1:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="44"/>
-      <c r="B14" s="44"/>
-      <c r="C14" s="45"/>
-      <c r="D14" s="49"/>
-      <c r="E14" s="50"/>
-      <c r="F14" s="135"/>
-      <c r="G14" s="136"/>
-      <c r="H14" s="56"/>
-      <c r="I14" s="59"/>
+      <c r="A14" s="79"/>
+      <c r="B14" s="79"/>
+      <c r="C14" s="80"/>
+      <c r="D14" s="84"/>
+      <c r="E14" s="85"/>
+      <c r="F14" s="158"/>
+      <c r="G14" s="159"/>
+      <c r="H14" s="91"/>
+      <c r="I14" s="94"/>
     </row>
     <row r="15" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="46"/>
-      <c r="B15" s="46"/>
-      <c r="C15" s="47"/>
-      <c r="D15" s="51"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="137"/>
-      <c r="G15" s="138"/>
-      <c r="H15" s="57"/>
-      <c r="I15" s="60"/>
+      <c r="A15" s="81"/>
+      <c r="B15" s="81"/>
+      <c r="C15" s="82"/>
+      <c r="D15" s="86"/>
+      <c r="E15" s="87"/>
+      <c r="F15" s="160"/>
+      <c r="G15" s="161"/>
+      <c r="H15" s="92"/>
+      <c r="I15" s="95"/>
     </row>
     <row r="16" spans="1:9" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="72" t="s">
+      <c r="A16" s="107" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="72"/>
-      <c r="C16" s="72"/>
-      <c r="D16" s="73"/>
-      <c r="E16" s="76" t="s">
+      <c r="B16" s="107"/>
+      <c r="C16" s="107"/>
+      <c r="D16" s="108"/>
+      <c r="E16" s="111" t="s">
         <v>7</v>
       </c>
-      <c r="F16" s="73"/>
-      <c r="G16" s="76" t="s">
+      <c r="F16" s="108"/>
+      <c r="G16" s="111" t="s">
         <v>8</v>
       </c>
-      <c r="H16" s="72"/>
-      <c r="I16" s="73"/>
+      <c r="H16" s="107"/>
+      <c r="I16" s="108"/>
     </row>
     <row r="17" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="74"/>
-      <c r="B17" s="74"/>
-      <c r="C17" s="74"/>
-      <c r="D17" s="75"/>
-      <c r="E17" s="77"/>
-      <c r="F17" s="75"/>
-      <c r="G17" s="77"/>
-      <c r="H17" s="74"/>
-      <c r="I17" s="75"/>
+      <c r="A17" s="109"/>
+      <c r="B17" s="109"/>
+      <c r="C17" s="109"/>
+      <c r="D17" s="110"/>
+      <c r="E17" s="112"/>
+      <c r="F17" s="110"/>
+      <c r="G17" s="112"/>
+      <c r="H17" s="109"/>
+      <c r="I17" s="110"/>
     </row>
     <row r="18" spans="1:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="41" t="s">
+      <c r="A18" s="76" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="41"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="78"/>
-      <c r="E18" s="80" t="s">
+      <c r="B18" s="76"/>
+      <c r="C18" s="76"/>
+      <c r="D18" s="113"/>
+      <c r="E18" s="115" t="s">
         <v>33</v>
       </c>
-      <c r="F18" s="78"/>
-      <c r="G18" s="80" t="s">
+      <c r="F18" s="113"/>
+      <c r="G18" s="115" t="s">
         <v>34</v>
       </c>
-      <c r="H18" s="41"/>
-      <c r="I18" s="78"/>
+      <c r="H18" s="76"/>
+      <c r="I18" s="113"/>
     </row>
     <row r="19" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="79"/>
-      <c r="B19" s="79"/>
-      <c r="C19" s="79"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="81"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="82"/>
-      <c r="H19" s="83"/>
-      <c r="I19" s="84"/>
+      <c r="A19" s="114"/>
+      <c r="B19" s="114"/>
+      <c r="C19" s="114"/>
+      <c r="D19" s="59"/>
+      <c r="E19" s="116"/>
+      <c r="F19" s="59"/>
+      <c r="G19" s="117"/>
+      <c r="H19" s="118"/>
+      <c r="I19" s="119"/>
     </row>
     <row r="20" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="61" t="s">
+      <c r="A20" s="96" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="61"/>
-      <c r="C20" s="61"/>
-      <c r="D20" s="61"/>
-      <c r="E20" s="61"/>
-      <c r="F20" s="61"/>
-      <c r="G20" s="62"/>
-      <c r="H20" s="63" t="s">
+      <c r="B20" s="96"/>
+      <c r="C20" s="96"/>
+      <c r="D20" s="96"/>
+      <c r="E20" s="96"/>
+      <c r="F20" s="96"/>
+      <c r="G20" s="97"/>
+      <c r="H20" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="I20" s="64"/>
+      <c r="I20" s="99"/>
     </row>
     <row r="21" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="65" t="s">
+      <c r="A21" s="100" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="66"/>
-      <c r="C21" s="66"/>
-      <c r="D21" s="66"/>
-      <c r="E21" s="66"/>
-      <c r="F21" s="66"/>
-      <c r="G21" s="67"/>
-      <c r="H21" s="139" t="s">
+      <c r="B21" s="101"/>
+      <c r="C21" s="101"/>
+      <c r="D21" s="101"/>
+      <c r="E21" s="101"/>
+      <c r="F21" s="101"/>
+      <c r="G21" s="102"/>
+      <c r="H21" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="I21" s="140"/>
+      <c r="I21" s="16"/>
     </row>
     <row r="22" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="68"/>
-      <c r="B22" s="68"/>
-      <c r="C22" s="68"/>
-      <c r="D22" s="68"/>
-      <c r="E22" s="68"/>
-      <c r="F22" s="68"/>
-      <c r="G22" s="69"/>
-      <c r="H22" s="141"/>
-      <c r="I22" s="142"/>
+      <c r="A22" s="103"/>
+      <c r="B22" s="103"/>
+      <c r="C22" s="103"/>
+      <c r="D22" s="103"/>
+      <c r="E22" s="103"/>
+      <c r="F22" s="103"/>
+      <c r="G22" s="104"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="18"/>
     </row>
     <row r="23" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="68"/>
-      <c r="B23" s="68"/>
-      <c r="C23" s="68"/>
-      <c r="D23" s="68"/>
-      <c r="E23" s="68"/>
-      <c r="F23" s="68"/>
-      <c r="G23" s="69"/>
-      <c r="H23" s="141"/>
-      <c r="I23" s="142"/>
+      <c r="A23" s="103"/>
+      <c r="B23" s="103"/>
+      <c r="C23" s="103"/>
+      <c r="D23" s="103"/>
+      <c r="E23" s="103"/>
+      <c r="F23" s="103"/>
+      <c r="G23" s="104"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="18"/>
     </row>
     <row r="24" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="68"/>
-      <c r="B24" s="68"/>
-      <c r="C24" s="68"/>
-      <c r="D24" s="68"/>
-      <c r="E24" s="68"/>
-      <c r="F24" s="68"/>
-      <c r="G24" s="69"/>
-      <c r="H24" s="141"/>
-      <c r="I24" s="142"/>
+      <c r="A24" s="103"/>
+      <c r="B24" s="103"/>
+      <c r="C24" s="103"/>
+      <c r="D24" s="103"/>
+      <c r="E24" s="103"/>
+      <c r="F24" s="103"/>
+      <c r="G24" s="104"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="18"/>
     </row>
     <row r="25" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="68"/>
-      <c r="B25" s="68"/>
-      <c r="C25" s="68"/>
-      <c r="D25" s="68"/>
-      <c r="E25" s="68"/>
-      <c r="F25" s="68"/>
-      <c r="G25" s="69"/>
-      <c r="H25" s="141"/>
-      <c r="I25" s="142"/>
+      <c r="A25" s="103"/>
+      <c r="B25" s="103"/>
+      <c r="C25" s="103"/>
+      <c r="D25" s="103"/>
+      <c r="E25" s="103"/>
+      <c r="F25" s="103"/>
+      <c r="G25" s="104"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="18"/>
     </row>
     <row r="26" spans="1:9" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="68"/>
-      <c r="B26" s="68"/>
-      <c r="C26" s="68"/>
-      <c r="D26" s="68"/>
-      <c r="E26" s="68"/>
-      <c r="F26" s="68"/>
-      <c r="G26" s="69"/>
-      <c r="H26" s="141"/>
-      <c r="I26" s="142"/>
+      <c r="A26" s="103"/>
+      <c r="B26" s="103"/>
+      <c r="C26" s="103"/>
+      <c r="D26" s="103"/>
+      <c r="E26" s="103"/>
+      <c r="F26" s="103"/>
+      <c r="G26" s="104"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="18"/>
     </row>
     <row r="27" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="68"/>
-      <c r="B27" s="68"/>
-      <c r="C27" s="68"/>
-      <c r="D27" s="68"/>
-      <c r="E27" s="68"/>
-      <c r="F27" s="68"/>
-      <c r="G27" s="69"/>
-      <c r="H27" s="141"/>
-      <c r="I27" s="142"/>
+      <c r="A27" s="103"/>
+      <c r="B27" s="103"/>
+      <c r="C27" s="103"/>
+      <c r="D27" s="103"/>
+      <c r="E27" s="103"/>
+      <c r="F27" s="103"/>
+      <c r="G27" s="104"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="18"/>
     </row>
     <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="70"/>
-      <c r="B28" s="70"/>
-      <c r="C28" s="70"/>
-      <c r="D28" s="70"/>
-      <c r="E28" s="70"/>
-      <c r="F28" s="70"/>
-      <c r="G28" s="71"/>
-      <c r="H28" s="143"/>
-      <c r="I28" s="144"/>
+      <c r="A28" s="105"/>
+      <c r="B28" s="105"/>
+      <c r="C28" s="105"/>
+      <c r="D28" s="105"/>
+      <c r="E28" s="105"/>
+      <c r="F28" s="105"/>
+      <c r="G28" s="106"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="20"/>
     </row>
     <row r="29" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="99" t="s">
+      <c r="A29" s="126" t="s">
         <v>11</v>
       </c>
-      <c r="B29" s="99"/>
-      <c r="C29" s="99"/>
-      <c r="D29" s="99"/>
-      <c r="E29" s="99"/>
-      <c r="F29" s="99"/>
-      <c r="G29" s="100"/>
+      <c r="B29" s="126"/>
+      <c r="C29" s="126"/>
+      <c r="D29" s="126"/>
+      <c r="E29" s="126"/>
+      <c r="F29" s="126"/>
+      <c r="G29" s="127"/>
       <c r="H29" s="7" t="s">
         <v>12</v>
       </c>
@@ -3279,379 +3312,411 @@
       </c>
     </row>
     <row r="30" spans="1:9" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="65" t="s">
+      <c r="A30" s="100" t="s">
         <v>43</v>
       </c>
-      <c r="B30" s="66"/>
-      <c r="C30" s="66"/>
-      <c r="D30" s="66"/>
-      <c r="E30" s="66"/>
-      <c r="F30" s="66"/>
-      <c r="G30" s="67"/>
-      <c r="H30" s="145" t="s">
+      <c r="B30" s="101"/>
+      <c r="C30" s="101"/>
+      <c r="D30" s="101"/>
+      <c r="E30" s="101"/>
+      <c r="F30" s="101"/>
+      <c r="G30" s="102"/>
+      <c r="H30" s="162" t="s">
         <v>44</v>
       </c>
-      <c r="I30" s="145" t="s">
+      <c r="I30" s="162" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="70"/>
-      <c r="B31" s="70"/>
-      <c r="C31" s="70"/>
-      <c r="D31" s="70"/>
-      <c r="E31" s="70"/>
-      <c r="F31" s="70"/>
-      <c r="G31" s="71"/>
-      <c r="H31" s="146"/>
-      <c r="I31" s="146"/>
+      <c r="A31" s="105"/>
+      <c r="B31" s="105"/>
+      <c r="C31" s="105"/>
+      <c r="D31" s="105"/>
+      <c r="E31" s="105"/>
+      <c r="F31" s="105"/>
+      <c r="G31" s="106"/>
+      <c r="H31" s="163"/>
+      <c r="I31" s="163"/>
     </row>
     <row r="32" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="101" t="s">
+      <c r="A32" s="128" t="s">
         <v>14</v>
       </c>
-      <c r="B32" s="101"/>
-      <c r="C32" s="101"/>
-      <c r="D32" s="101"/>
-      <c r="E32" s="101"/>
-      <c r="F32" s="101"/>
-      <c r="G32" s="101"/>
-      <c r="H32" s="102"/>
+      <c r="B32" s="128"/>
+      <c r="C32" s="128"/>
+      <c r="D32" s="128"/>
+      <c r="E32" s="128"/>
+      <c r="F32" s="128"/>
+      <c r="G32" s="128"/>
+      <c r="H32" s="129"/>
       <c r="I32" s="9" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="103" t="s">
+      <c r="A33" s="130" t="s">
         <v>47</v>
       </c>
-      <c r="B33" s="103"/>
-      <c r="C33" s="103"/>
-      <c r="D33" s="103"/>
-      <c r="E33" s="103"/>
-      <c r="F33" s="103"/>
-      <c r="G33" s="103"/>
-      <c r="H33" s="104"/>
+      <c r="B33" s="130"/>
+      <c r="C33" s="130"/>
+      <c r="D33" s="130"/>
+      <c r="E33" s="130"/>
+      <c r="F33" s="130"/>
+      <c r="G33" s="130"/>
+      <c r="H33" s="131"/>
       <c r="I33" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="105"/>
-      <c r="B34" s="105"/>
-      <c r="C34" s="105"/>
-      <c r="D34" s="105"/>
-      <c r="E34" s="105"/>
-      <c r="F34" s="105"/>
-      <c r="G34" s="105"/>
-      <c r="H34" s="106"/>
-      <c r="I34" s="85" t="s">
+      <c r="A34" s="132"/>
+      <c r="B34" s="132"/>
+      <c r="C34" s="132"/>
+      <c r="D34" s="132"/>
+      <c r="E34" s="132"/>
+      <c r="F34" s="132"/>
+      <c r="G34" s="132"/>
+      <c r="H34" s="133"/>
+      <c r="I34" s="164" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="107"/>
-      <c r="B35" s="107"/>
-      <c r="C35" s="107"/>
-      <c r="D35" s="107"/>
-      <c r="E35" s="107"/>
-      <c r="F35" s="107"/>
-      <c r="G35" s="107"/>
-      <c r="H35" s="108"/>
-      <c r="I35" s="86"/>
+      <c r="A35" s="134"/>
+      <c r="B35" s="134"/>
+      <c r="C35" s="134"/>
+      <c r="D35" s="134"/>
+      <c r="E35" s="134"/>
+      <c r="F35" s="134"/>
+      <c r="G35" s="134"/>
+      <c r="H35" s="135"/>
+      <c r="I35" s="165"/>
     </row>
     <row r="36" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="A36" s="109" t="s">
+      <c r="A36" s="136" t="s">
         <v>17</v>
       </c>
-      <c r="B36" s="110"/>
-      <c r="C36" s="110"/>
-      <c r="D36" s="110"/>
-      <c r="E36" s="111"/>
-      <c r="F36" s="112" t="s">
+      <c r="B36" s="137"/>
+      <c r="C36" s="137"/>
+      <c r="D36" s="137"/>
+      <c r="E36" s="138"/>
+      <c r="F36" s="139" t="s">
         <v>18</v>
       </c>
-      <c r="G36" s="113"/>
-      <c r="H36" s="113"/>
-      <c r="I36" s="114"/>
+      <c r="G36" s="140"/>
+      <c r="H36" s="140"/>
+      <c r="I36" s="141"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A37" s="115" t="s">
+      <c r="A37" s="142" t="s">
         <v>19</v>
       </c>
-      <c r="B37" s="116"/>
-      <c r="C37" s="116"/>
-      <c r="D37" s="116"/>
-      <c r="E37" s="117"/>
-      <c r="F37" s="118" t="s">
+      <c r="B37" s="143"/>
+      <c r="C37" s="143"/>
+      <c r="D37" s="143"/>
+      <c r="E37" s="144"/>
+      <c r="F37" s="145" t="s">
         <v>20</v>
       </c>
-      <c r="G37" s="119"/>
-      <c r="H37" s="119"/>
-      <c r="I37" s="120"/>
+      <c r="G37" s="146"/>
+      <c r="H37" s="146"/>
+      <c r="I37" s="147"/>
     </row>
     <row r="38" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="147" t="s">
+      <c r="A38" s="166" t="s">
         <v>49</v>
       </c>
-      <c r="B38" s="147"/>
-      <c r="C38" s="147"/>
-      <c r="D38" s="147"/>
-      <c r="E38" s="148"/>
-      <c r="F38" s="153" t="s">
+      <c r="B38" s="166"/>
+      <c r="C38" s="166"/>
+      <c r="D38" s="166"/>
+      <c r="E38" s="167"/>
+      <c r="F38" s="172" t="s">
         <v>50</v>
       </c>
-      <c r="G38" s="147"/>
-      <c r="H38" s="147"/>
-      <c r="I38" s="148"/>
+      <c r="G38" s="166"/>
+      <c r="H38" s="166"/>
+      <c r="I38" s="167"/>
     </row>
     <row r="39" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="149"/>
-      <c r="B39" s="149"/>
-      <c r="C39" s="149"/>
-      <c r="D39" s="149"/>
-      <c r="E39" s="150"/>
-      <c r="F39" s="154"/>
-      <c r="G39" s="149"/>
-      <c r="H39" s="149"/>
-      <c r="I39" s="150"/>
+      <c r="A39" s="168"/>
+      <c r="B39" s="168"/>
+      <c r="C39" s="168"/>
+      <c r="D39" s="168"/>
+      <c r="E39" s="169"/>
+      <c r="F39" s="173"/>
+      <c r="G39" s="168"/>
+      <c r="H39" s="168"/>
+      <c r="I39" s="169"/>
     </row>
     <row r="40" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="149"/>
-      <c r="B40" s="149"/>
-      <c r="C40" s="149"/>
-      <c r="D40" s="149"/>
-      <c r="E40" s="150"/>
-      <c r="F40" s="154"/>
-      <c r="G40" s="149"/>
-      <c r="H40" s="149"/>
-      <c r="I40" s="150"/>
+      <c r="A40" s="168"/>
+      <c r="B40" s="168"/>
+      <c r="C40" s="168"/>
+      <c r="D40" s="168"/>
+      <c r="E40" s="169"/>
+      <c r="F40" s="173"/>
+      <c r="G40" s="168"/>
+      <c r="H40" s="168"/>
+      <c r="I40" s="169"/>
     </row>
     <row r="41" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="149"/>
-      <c r="B41" s="149"/>
-      <c r="C41" s="149"/>
-      <c r="D41" s="149"/>
-      <c r="E41" s="150"/>
-      <c r="F41" s="154"/>
-      <c r="G41" s="149"/>
-      <c r="H41" s="149"/>
-      <c r="I41" s="150"/>
+      <c r="A41" s="168"/>
+      <c r="B41" s="168"/>
+      <c r="C41" s="168"/>
+      <c r="D41" s="168"/>
+      <c r="E41" s="169"/>
+      <c r="F41" s="173"/>
+      <c r="G41" s="168"/>
+      <c r="H41" s="168"/>
+      <c r="I41" s="169"/>
     </row>
     <row r="42" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="149"/>
-      <c r="B42" s="149"/>
-      <c r="C42" s="149"/>
-      <c r="D42" s="149"/>
-      <c r="E42" s="150"/>
-      <c r="F42" s="154"/>
-      <c r="G42" s="149"/>
-      <c r="H42" s="149"/>
-      <c r="I42" s="150"/>
+      <c r="A42" s="168"/>
+      <c r="B42" s="168"/>
+      <c r="C42" s="168"/>
+      <c r="D42" s="168"/>
+      <c r="E42" s="169"/>
+      <c r="F42" s="173"/>
+      <c r="G42" s="168"/>
+      <c r="H42" s="168"/>
+      <c r="I42" s="169"/>
     </row>
     <row r="43" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="149"/>
-      <c r="B43" s="149"/>
-      <c r="C43" s="149"/>
-      <c r="D43" s="149"/>
-      <c r="E43" s="150"/>
-      <c r="F43" s="154"/>
-      <c r="G43" s="149"/>
-      <c r="H43" s="149"/>
-      <c r="I43" s="150"/>
+      <c r="A43" s="168"/>
+      <c r="B43" s="168"/>
+      <c r="C43" s="168"/>
+      <c r="D43" s="168"/>
+      <c r="E43" s="169"/>
+      <c r="F43" s="173"/>
+      <c r="G43" s="168"/>
+      <c r="H43" s="168"/>
+      <c r="I43" s="169"/>
     </row>
     <row r="44" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="149"/>
-      <c r="B44" s="149"/>
-      <c r="C44" s="149"/>
-      <c r="D44" s="149"/>
-      <c r="E44" s="150"/>
-      <c r="F44" s="154"/>
-      <c r="G44" s="149"/>
-      <c r="H44" s="149"/>
-      <c r="I44" s="150"/>
+      <c r="A44" s="168"/>
+      <c r="B44" s="168"/>
+      <c r="C44" s="168"/>
+      <c r="D44" s="168"/>
+      <c r="E44" s="169"/>
+      <c r="F44" s="173"/>
+      <c r="G44" s="168"/>
+      <c r="H44" s="168"/>
+      <c r="I44" s="169"/>
     </row>
     <row r="45" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="149"/>
-      <c r="B45" s="149"/>
-      <c r="C45" s="149"/>
-      <c r="D45" s="149"/>
-      <c r="E45" s="150"/>
-      <c r="F45" s="154"/>
-      <c r="G45" s="149"/>
-      <c r="H45" s="149"/>
-      <c r="I45" s="150"/>
+      <c r="A45" s="168"/>
+      <c r="B45" s="168"/>
+      <c r="C45" s="168"/>
+      <c r="D45" s="168"/>
+      <c r="E45" s="169"/>
+      <c r="F45" s="173"/>
+      <c r="G45" s="168"/>
+      <c r="H45" s="168"/>
+      <c r="I45" s="169"/>
     </row>
     <row r="46" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="151"/>
-      <c r="B46" s="151"/>
-      <c r="C46" s="151"/>
-      <c r="D46" s="151"/>
-      <c r="E46" s="152"/>
-      <c r="F46" s="155"/>
-      <c r="G46" s="151"/>
-      <c r="H46" s="151"/>
-      <c r="I46" s="152"/>
+      <c r="A46" s="170"/>
+      <c r="B46" s="170"/>
+      <c r="C46" s="170"/>
+      <c r="D46" s="170"/>
+      <c r="E46" s="171"/>
+      <c r="F46" s="174"/>
+      <c r="G46" s="170"/>
+      <c r="H46" s="170"/>
+      <c r="I46" s="171"/>
     </row>
     <row r="47" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="156" t="s">
+      <c r="A47" s="175" t="s">
         <v>21</v>
       </c>
-      <c r="B47" s="156"/>
-      <c r="C47" s="156"/>
-      <c r="D47" s="156"/>
-      <c r="E47" s="156"/>
-      <c r="F47" s="156"/>
-      <c r="G47" s="156"/>
-      <c r="H47" s="156"/>
-      <c r="I47" s="157"/>
+      <c r="B47" s="175"/>
+      <c r="C47" s="175"/>
+      <c r="D47" s="175"/>
+      <c r="E47" s="175"/>
+      <c r="F47" s="175"/>
+      <c r="G47" s="175"/>
+      <c r="H47" s="175"/>
+      <c r="I47" s="176"/>
     </row>
     <row r="48" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="121" t="s">
+      <c r="A48" s="148" t="s">
         <v>22</v>
       </c>
-      <c r="B48" s="122"/>
-      <c r="C48" s="122"/>
-      <c r="D48" s="122"/>
-      <c r="E48" s="122"/>
-      <c r="F48" s="122"/>
-      <c r="G48" s="123"/>
-      <c r="H48" s="10" t="s">
+      <c r="B48" s="149"/>
+      <c r="C48" s="149"/>
+      <c r="D48" s="149"/>
+      <c r="E48" s="149"/>
+      <c r="F48" s="149"/>
+      <c r="G48" s="150"/>
+      <c r="H48" s="151" t="s">
         <v>13</v>
       </c>
-      <c r="I48" s="11" t="s">
+      <c r="I48" s="152"/>
+    </row>
+    <row r="49" spans="1:9" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="42" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" s="42"/>
+      <c r="C49" s="42"/>
+      <c r="D49" s="42"/>
+      <c r="E49" s="42"/>
+      <c r="F49" s="42"/>
+      <c r="G49" s="43"/>
+      <c r="H49" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="I49" s="16"/>
+    </row>
+    <row r="50" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="44"/>
+      <c r="B50" s="44"/>
+      <c r="C50" s="44"/>
+      <c r="D50" s="44"/>
+      <c r="E50" s="44"/>
+      <c r="F50" s="44"/>
+      <c r="G50" s="45"/>
+      <c r="H50" s="178" t="s">
+        <v>55</v>
+      </c>
+      <c r="I50" s="178"/>
+    </row>
+    <row r="51" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="46"/>
+      <c r="B51" s="46"/>
+      <c r="C51" s="46"/>
+      <c r="D51" s="46"/>
+      <c r="E51" s="46"/>
+      <c r="F51" s="46"/>
+      <c r="G51" s="47"/>
+      <c r="H51" s="178" t="s">
+        <v>54</v>
+      </c>
+      <c r="I51" s="178"/>
+    </row>
+    <row r="52" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="120" t="s">
+        <v>23</v>
+      </c>
+      <c r="B52" s="121"/>
+      <c r="C52" s="122"/>
+      <c r="D52" s="123" t="s">
+        <v>24</v>
+      </c>
+      <c r="E52" s="124"/>
+      <c r="F52" s="125"/>
+      <c r="G52" s="10" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="93" t="s">
-        <v>48</v>
-      </c>
-      <c r="B49" s="94"/>
-      <c r="C49" s="94"/>
-      <c r="D49" s="94"/>
-      <c r="E49" s="94"/>
-      <c r="F49" s="94"/>
-      <c r="G49" s="95"/>
-      <c r="H49" s="145" t="s">
-        <v>45</v>
-      </c>
-      <c r="I49" s="85" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="96"/>
-      <c r="B50" s="97"/>
-      <c r="C50" s="97"/>
-      <c r="D50" s="97"/>
-      <c r="E50" s="97"/>
-      <c r="F50" s="97"/>
-      <c r="G50" s="98"/>
-      <c r="H50" s="146"/>
-      <c r="I50" s="86"/>
-    </row>
-    <row r="51" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="87" t="s">
-        <v>23</v>
-      </c>
-      <c r="B51" s="88"/>
-      <c r="C51" s="89"/>
-      <c r="D51" s="90" t="s">
-        <v>24</v>
-      </c>
-      <c r="E51" s="91"/>
-      <c r="F51" s="92"/>
-      <c r="G51" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H51" s="12" t="s">
+      <c r="H52" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="I51" s="12" t="s">
+      <c r="I52" s="11" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="126" t="s">
+    <row r="53" spans="1:9" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="B52" s="126"/>
-      <c r="C52" s="127"/>
-      <c r="D52" s="131"/>
-      <c r="E52" s="126"/>
-      <c r="F52" s="127"/>
-      <c r="G52" s="145"/>
-      <c r="H52" s="145"/>
-      <c r="I52" s="85" t="s">
+      <c r="B53" s="33"/>
+      <c r="C53" s="34"/>
+      <c r="D53" s="39"/>
+      <c r="E53" s="33"/>
+      <c r="F53" s="34"/>
+      <c r="G53" s="13"/>
+      <c r="H53" s="14"/>
+      <c r="I53" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="128"/>
-      <c r="B53" s="128"/>
-      <c r="C53" s="129"/>
-      <c r="D53" s="132"/>
-      <c r="E53" s="128"/>
-      <c r="F53" s="129"/>
-      <c r="G53" s="146"/>
-      <c r="H53" s="146"/>
-      <c r="I53" s="86"/>
-    </row>
-    <row r="54" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="130" t="s">
+    <row r="54" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="35"/>
+      <c r="B54" s="35"/>
+      <c r="C54" s="36"/>
+      <c r="D54" s="40"/>
+      <c r="E54" s="35"/>
+      <c r="F54" s="36"/>
+      <c r="G54" s="177" t="s">
+        <v>55</v>
+      </c>
+      <c r="H54" s="177" t="s">
+        <v>55</v>
+      </c>
+      <c r="I54" s="177" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="37"/>
+      <c r="B55" s="37"/>
+      <c r="C55" s="38"/>
+      <c r="D55" s="41"/>
+      <c r="E55" s="37"/>
+      <c r="F55" s="38"/>
+      <c r="G55" s="177" t="s">
+        <v>54</v>
+      </c>
+      <c r="H55" s="177" t="s">
+        <v>54</v>
+      </c>
+      <c r="I55" s="177" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="155" t="s">
         <v>27</v>
       </c>
-      <c r="B54" s="130"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
-      <c r="I54" s="5"/>
-    </row>
-    <row r="55" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="124" t="s">
+      <c r="B56" s="155"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="I56" s="5"/>
+    </row>
+    <row r="57" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="153" t="s">
         <v>51</v>
       </c>
-      <c r="B55" s="124"/>
-      <c r="C55" s="124"/>
-      <c r="D55" s="124"/>
-      <c r="E55" s="124"/>
-      <c r="F55" s="124"/>
-      <c r="G55" s="124"/>
-      <c r="H55" s="124"/>
-      <c r="I55" s="3"/>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A56" s="124"/>
-      <c r="B56" s="124"/>
-      <c r="C56" s="124"/>
-      <c r="D56" s="124"/>
-      <c r="E56" s="124"/>
-      <c r="F56" s="124"/>
-      <c r="G56" s="124"/>
-      <c r="H56" s="124"/>
-      <c r="I56" s="3"/>
-    </row>
-    <row r="57" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="125"/>
-      <c r="B57" s="125"/>
-      <c r="C57" s="125"/>
-      <c r="D57" s="125"/>
-      <c r="E57" s="125"/>
-      <c r="F57" s="125"/>
-      <c r="G57" s="125"/>
-      <c r="H57" s="125"/>
-      <c r="I57" s="4"/>
-    </row>
-    <row r="58" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="59" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="60" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="B57" s="153"/>
+      <c r="C57" s="153"/>
+      <c r="D57" s="153"/>
+      <c r="E57" s="153"/>
+      <c r="F57" s="153"/>
+      <c r="G57" s="153"/>
+      <c r="H57" s="153"/>
+      <c r="I57" s="3"/>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A58" s="153"/>
+      <c r="B58" s="153"/>
+      <c r="C58" s="153"/>
+      <c r="D58" s="153"/>
+      <c r="E58" s="153"/>
+      <c r="F58" s="153"/>
+      <c r="G58" s="153"/>
+      <c r="H58" s="153"/>
+      <c r="I58" s="3"/>
+    </row>
+    <row r="59" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="154"/>
+      <c r="B59" s="154"/>
+      <c r="C59" s="154"/>
+      <c r="D59" s="154"/>
+      <c r="E59" s="154"/>
+      <c r="F59" s="154"/>
+      <c r="G59" s="154"/>
+      <c r="H59" s="154"/>
+      <c r="I59" s="4"/>
+    </row>
+    <row r="60" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="61" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="62" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="55">
-    <mergeCell ref="A55:H57"/>
-    <mergeCell ref="A52:C53"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="D52:F53"/>
+  <mergeCells count="54">
+    <mergeCell ref="A57:H59"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="F11:G15"/>
     <mergeCell ref="H21:I28"/>
     <mergeCell ref="H30:H31"/>
@@ -3660,14 +3725,8 @@
     <mergeCell ref="A38:E46"/>
     <mergeCell ref="F38:I46"/>
     <mergeCell ref="A47:I47"/>
-    <mergeCell ref="G52:G53"/>
-    <mergeCell ref="H52:H53"/>
-    <mergeCell ref="I52:I53"/>
-    <mergeCell ref="H49:H50"/>
-    <mergeCell ref="I49:I50"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="A49:G50"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="D52:F52"/>
     <mergeCell ref="A29:G29"/>
     <mergeCell ref="A30:G31"/>
     <mergeCell ref="A32:H32"/>
@@ -3677,6 +3736,30 @@
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="F37:I37"/>
     <mergeCell ref="A48:G48"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="A53:C55"/>
+    <mergeCell ref="D53:F55"/>
+    <mergeCell ref="A49:G51"/>
+    <mergeCell ref="F1:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="A9:C10"/>
+    <mergeCell ref="D9:E10"/>
+    <mergeCell ref="F9:G10"/>
+    <mergeCell ref="H9:I10"/>
+    <mergeCell ref="A11:C15"/>
+    <mergeCell ref="D11:E15"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="H49:I49"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="H51:I51"/>
+    <mergeCell ref="A1:C8"/>
+    <mergeCell ref="D1:E8"/>
+    <mergeCell ref="H13:H15"/>
+    <mergeCell ref="I13:I15"/>
     <mergeCell ref="A20:G20"/>
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="A21:G28"/>
@@ -3686,23 +3769,6 @@
     <mergeCell ref="A18:D19"/>
     <mergeCell ref="E18:F19"/>
     <mergeCell ref="G18:I19"/>
-    <mergeCell ref="A9:C10"/>
-    <mergeCell ref="D9:E10"/>
-    <mergeCell ref="F9:G10"/>
-    <mergeCell ref="H9:I10"/>
-    <mergeCell ref="A11:C15"/>
-    <mergeCell ref="D11:E15"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="H13:H15"/>
-    <mergeCell ref="I13:I15"/>
-    <mergeCell ref="F1:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I8"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="A1:C8"/>
-    <mergeCell ref="D1:E8"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>